<commit_message>
creacion de carga masiva para libros
</commit_message>
<xml_diff>
--- a/docs/Casos de Prueba Web/Casos de Prueba_Web.xlsx
+++ b/docs/Casos de Prueba Web/Casos de Prueba_Web.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jbeto\OneDrive\Escritorio\C-book-Proyecto\docs\Casos de Prueba Web\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F35BD537-6649-4062-8834-46AAC46D2970}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA593BDA-A1E4-4A6A-B9C2-A9DD6A189451}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -95,16 +95,6 @@
     <t>Principal</t>
   </si>
   <si>
-    <t>Precondiciones: Boleta autorizada sin cuenta y correo institucional disponible
-1- Abrir / 
-2- Cambiar a modo registro
-3- Ingresar boleta valida
-4- Ingresar correo @alumno.ipn.mx
-5- Ingresar contrasena valida
-6- Confirmar contrasena
-7- Pulsar Registrarse</t>
-  </si>
-  <si>
     <t>Boleta: 10 digitos
 Correo: @alumno.ipn.mx
 Contrasena: 6-16, minuscula, mayuscula y especial
@@ -231,13 +221,6 @@
     <t>Login de alumno correcto</t>
   </si>
   <si>
-    <t>Precondiciones: Alumno registrado y verificado
-1- Abrir /
-2- Ingresar boleta
-3- Ingresar contrasena
-4- Pulsar Iniciar sesion</t>
-  </si>
-  <si>
     <t>Boleta 10 digitos
 Password obligatorio</t>
   </si>
@@ -256,13 +239,6 @@
   </si>
   <si>
     <t>Login Admin correcto</t>
-  </si>
-  <si>
-    <t>Precondiciones: Cuenta Admin existente
-1- Abrir /
-2- Ingresar boleta admin
-3- Ingresar password
-4- Pulsar Iniciar sesion</t>
   </si>
   <si>
     <t>Rol devuelto debe ser Admin</t>
@@ -309,13 +285,6 @@
     <t>Login de soporte correcto</t>
   </si>
   <si>
-    <t>Precondiciones: Cuenta support_admin o support_agent activa
-1- Abrir login
-2- Ingresar identificador de soporte
-3- Ingresar password
-4- Pulsar Iniciar sesion</t>
-  </si>
-  <si>
     <t>Perfil soporte activo
 Rol support_admin/support_agent</t>
   </si>
@@ -345,13 +314,6 @@
     <t>Activacion posterior a confirmacion</t>
   </si>
   <si>
-    <t>Precondiciones: Alumno registrado y correo confirmado en Supabase Auth
-1- Abrir enlace de verificacion
-2- Entrar a /verificar
-3- El frontend envia boleta y correo
-4- Observar resultado</t>
-  </si>
-  <si>
     <t>boleta y correo guardados del registro
 email_confirmed_at confirmado</t>
   </si>
@@ -372,12 +334,6 @@
     <t>Correo aun no confirmado</t>
   </si>
   <si>
-    <t>Precondiciones: Alumno registrado sin confirmar correo
-1- Registrar alumno
-2- No abrir correo
-3- Abrir /verificar o intentar verificar</t>
-  </si>
-  <si>
     <t>Supabase aun sin confirmacion</t>
   </si>
   <si>
@@ -403,16 +359,6 @@
   </si>
   <si>
     <t>Recuperar contrasena correctamente</t>
-  </si>
-  <si>
-    <t>Precondiciones: Boleta registrada con correo disponible
-1- Abrir /forgot-password
-2- Ingresar boleta
-3- Enviar enlace
-4- Abrir /reset-password?token=...
-5- Ingresar nueva contrasena
-6- Confirmar
-7- Guardar</t>
   </si>
   <si>
     <t>Boleta 10 digitos
@@ -461,11 +407,6 @@
     <t>Token ausente o invalido</t>
   </si>
   <si>
-    <t>Precondiciones: Abrir reset sin token valido
-1- Abrir /reset-password
-2- Observar mensaje</t>
-  </si>
-  <si>
     <t>Token requerido en query string</t>
   </si>
   <si>
@@ -493,12 +434,6 @@
     <t>Consulta de sesion activa</t>
   </si>
   <si>
-    <t>Precondiciones: Usuario autenticado con cookie app_session
-1- Iniciar sesion
-2- Recargar pagina
-3- AuthContext llama /auth/session</t>
-  </si>
-  <si>
     <t>Cookie valida y JWT verificable</t>
   </si>
   <si>
@@ -515,11 +450,6 @@
   </si>
   <si>
     <t>Acceso sin sesion a ruta protegida</t>
-  </si>
-  <si>
-    <t>Precondiciones: No tener cookie valida
-1- Abrir /admin
-2- Observar redireccion</t>
   </si>
   <si>
     <t>ProtectedRoute exige sesion y rol</t>
@@ -573,11 +503,6 @@
     <t>Ver perfil</t>
   </si>
   <si>
-    <t>Precondiciones: Usuario autenticado
-1- Ingresar a /user/perfil
-2- Observar datos y resumen</t>
-  </si>
-  <si>
     <t>Sesion activa</t>
   </si>
   <si>
@@ -594,14 +519,6 @@
   </si>
   <si>
     <t>Cambiar contrasena propia</t>
-  </si>
-  <si>
-    <t>Precondiciones: Usuario autenticado
-1- Ir a cuenta/perfil
-2- Capturar correo de sesion
-3- Capturar password actual
-4- Capturar nuevo password
-5- Guardar</t>
   </si>
   <si>
     <t>Correo coincide con sesion
@@ -634,12 +551,6 @@
     <t>Visualizar libros</t>
   </si>
   <si>
-    <t>Precondiciones: Alumno autenticado
-1- Ir a /user/libros
-2- Esperar carga de recursos
-3- Revisar listado</t>
-  </si>
-  <si>
     <t>GET /auth/recursos?tipo=libro</t>
   </si>
   <si>
@@ -658,11 +569,6 @@
     <t>Fallo de carga</t>
   </si>
   <si>
-    <t>Precondiciones: Alumno autenticado y API no disponible
-1- Ir a /user/libros
-2- Simular error de backend</t>
-  </si>
-  <si>
     <t>Manejo de error en frontend</t>
   </si>
   <si>
@@ -688,13 +594,6 @@
   </si>
   <si>
     <t>Solicitar libro disponible</t>
-  </si>
-  <si>
-    <t>Precondiciones: Alumno con documentos habilitados y menos de 3 solicitudes activas
-1- Ir a /user/libros
-2- Seleccionar libro disponible
-3- Pulsar solicitar
-4- Confirmar modal</t>
   </si>
   <si>
     <t>tipo libro
@@ -720,11 +619,6 @@
     <t>Alumno sin documentacion</t>
   </si>
   <si>
-    <t>Precondiciones: Alumno tiene_documentos=false
-1- Ir a /user/libros
-2- Intentar solicitar libro</t>
-  </si>
-  <si>
     <t>Boleta sin documentos</t>
   </si>
   <si>
@@ -746,11 +640,6 @@
     <t>Limite de 3 solicitudes activas</t>
   </si>
   <si>
-    <t>Precondiciones: Alumno con 3 solicitudes activas
-1- Ir a /user/libros
-2- Intentar solicitar otro libro</t>
-  </si>
-  <si>
     <t>Maximo 3 solicitudes activas</t>
   </si>
   <si>
@@ -767,13 +656,6 @@
   </si>
   <si>
     <t>Cancelar solicitud</t>
-  </si>
-  <si>
-    <t>Precondiciones: Alumno con solicitud cancelable
-1- Ir a mis solicitudes
-2- Seleccionar solicitud pendiente
-3- Pulsar cancelar
-4- Confirmar</t>
   </si>
   <si>
     <t>Solicitud debe pertenecer al usuario y estar en estado cancelable</t>
@@ -802,13 +684,6 @@
   </si>
   <si>
     <t>Crear libro y ejemplar</t>
-  </si>
-  <si>
-    <t>Precondiciones: Admin autenticado
-1- Ir a /admin/libros
-2- Capturar datos de libro
-3- Capturar datos de ejemplar
-4- Guardar</t>
   </si>
   <si>
     <t>Campos requeridos
@@ -892,14 +767,6 @@
     <t>Crear boleta</t>
   </si>
   <si>
-    <t>Precondiciones: Admin autenticado
-1- Ir a /admin/alumnos
-2- Capturar boleta
-3- Capturar nombre
-4- Capturar grupo
-5- Guardar</t>
-  </si>
-  <si>
     <t>Boleta 10 digitos
 Nombre requerido
 Grupo formato valido</t>
@@ -945,12 +812,6 @@
     <t>Preview de Excel valido</t>
   </si>
   <si>
-    <t>Precondiciones: Admin autenticado con archivo XLSX
-1- Ir a carga masiva
-2- Seleccionar XLSX
-3- Enviar preview</t>
-  </si>
-  <si>
     <t>Archivo CSV/XLSX
 Columnas boleta, nombre, Grupo
 Filas clasificadas</t>
@@ -1003,12 +864,6 @@
     <t>Habilitar documentacion</t>
   </si>
   <si>
-    <t>Precondiciones: Admin autenticado y usuario existente
-1- Ir a /admin/documentos o usuarios
-2- Seleccionar alumno
-3- Habilitar documentacion</t>
-  </si>
-  <si>
     <t>id de usuario requerido</t>
   </si>
   <si>
@@ -1056,13 +911,6 @@
   </si>
   <si>
     <t>Aprobar solicitud</t>
-  </si>
-  <si>
-    <t>Precondiciones: Admin autenticado y alumno con documentos
-1- Ir a /admin/solicitudes-libros
-2- Seleccionar solicitud
-3- Elegir aprobar
-4- Confirmar</t>
   </si>
   <si>
     <t>estado=2
@@ -1113,13 +961,6 @@
     <t>Entregar libro</t>
   </si>
   <si>
-    <t>Precondiciones: Solicitud aprobada y ejemplar disponible
-1- Ir a solicitudes
-2- Seleccionar aprobada
-3- Registrar entrega
-4- Confirmar</t>
-  </si>
-  <si>
     <t>id requerido
 Alumno con documentos
 Ejemplar valido</t>
@@ -1148,11 +989,6 @@
   </si>
   <si>
     <t>Consultar prestamos</t>
-  </si>
-  <si>
-    <t>Precondiciones: Admin autenticado
-1- Ir a /admin/prestamos-libros
-2- Observar listado</t>
   </si>
   <si>
     <t>GET /auth/admin/prestamos/libros</t>
@@ -1209,11 +1045,6 @@
     <t>Ver estadisticas</t>
   </si>
   <si>
-    <t>Precondiciones: Admin autenticado
-1- Ir a /admin/analytics
-2- Esperar carga</t>
-  </si>
-  <si>
     <t>Sesion Admin
 Datos desde solicitudes_libros y prestamos_libros</t>
   </si>
@@ -1230,11 +1061,6 @@
     <t>Exportar reporte</t>
   </si>
   <si>
-    <t>Precondiciones: Admin autenticado con datos cargados
-1- Ir a reportes
-2- Seleccionar exportar PDF o Excel</t>
-  </si>
-  <si>
     <t>Datos cargados en UI
 Utilidades exportPDF/exportExcel</t>
   </si>
@@ -1261,14 +1087,6 @@
   </si>
   <si>
     <t>Crear ticket autenticado</t>
-  </si>
-  <si>
-    <t>Precondiciones: Usuario autenticado
-1- Abrir SupportFab
-2- Elegir reportar
-3- Seleccionar tipo
-4- Ingresar modulo, titulo y descripcion
-5- Enviar</t>
   </si>
   <si>
     <t>Descripcion obligatoria
@@ -1293,13 +1111,6 @@
   </si>
   <si>
     <t>Crear ticket publico</t>
-  </si>
-  <si>
-    <t>Precondiciones: Usuario sin sesion
-1- Abrir /soporte/reportar
-2- Capturar correo y nombre
-3- Completar incidencia
-4- Enviar</t>
   </si>
   <si>
     <t>Correo obligatorio y formato valido
@@ -1356,12 +1167,6 @@
     <t>Listar bandeja</t>
   </si>
   <si>
-    <t>Precondiciones: Usuario support_admin/support_agent autenticado
-1- Entrar a /soporte/tickets
-2- Aplicar filtros
-3- Observar resultados</t>
-  </si>
-  <si>
     <t>Rol soporte
 Filtros estado/tipo/prioridad/q</t>
   </si>
@@ -1489,15 +1294,6 @@
     <t>Crear agente de soporte</t>
   </si>
   <si>
-    <t>Precondiciones: Sesion support_admin
-1- Entrar a /soporte/agregar-agente
-2- Capturar nombre
-3- Capturar correo
-4- Capturar boleta opcional
-5- Capturar password y confirmacion
-6- Guardar</t>
-  </si>
-  <si>
     <t>Solo support_admin
 Nombre, correo y password obligatorios
 Confirmacion igual
@@ -1547,10 +1343,6 @@
     <t>Acceso de support_agent a crear agente</t>
   </si>
   <si>
-    <t>Precondiciones: Sesion support_agent
-1- Intentar abrir /soporte/agregar-agente o llamar POST /soporte/agentes</t>
-  </si>
-  <si>
     <t>Solo support_admin</t>
   </si>
   <si>
@@ -1561,6 +1353,102 @@
   </si>
   <si>
     <t>La cuenta support_agent fue redirigida a /soporte y no pudo entrar a la pantalla de crear agentes.</t>
+  </si>
+  <si>
+    <t>Precondiciones: Boleta autorizada sin cuenta y correo institucional disponible | 1- Abrir C-Book Web | 2- Hacer clic en Crear cuenta | 3- Ingresar boleta valida | 4- Ingresar correo @alumno.ipn.mx | 5- Ingresar contrasena valida | 6- Confirmar contrasena | 7- Pulsar REGISTRAR</t>
+  </si>
+  <si>
+    <t>Precondiciones: Alumno registrado y verificado | 1- Abrir C-Book Web | 2- Ingresar boleta | 3- Ingresar contrasena | 4- Pulsar ACCEDER</t>
+  </si>
+  <si>
+    <t>Precondiciones: Cuenta Admin existente | 1- Abrir C-Book Web | 2- Ingresar boleta admin | 3- Ingresar password | 4- Pulsar ACCEDER</t>
+  </si>
+  <si>
+    <t>Precondiciones: Cuenta support_admin o support_agent activa | 1- Abrir C-Book Web | 2- Ingresar identificador de soporte | 3- Ingresar password | 4- Pulsar ACCEDER</t>
+  </si>
+  <si>
+    <t>Precondiciones: Alumno registrado y correo confirmado en Supabase Auth | 1- Abrir el enlace de verificacion del correo | 2- Esperar la pantalla de verificacion | 3- Esperar que termine la validacion | 4- Observar resultado</t>
+  </si>
+  <si>
+    <t>Precondiciones: Alumno registrado sin confirmar correo | 1- Hacer clic en Crear cuenta | 2- Completar el registro | 3- No abrir el correo de verificacion | 4- Intentar completar la verificacion</t>
+  </si>
+  <si>
+    <t>Precondiciones: Boleta registrada con correo disponible | 1- Hacer clic en Olvidaste tu contrasena? | 2- Ingresar boleta | 3- Pulsar ENVIAR ENLACE | 4- Abrir el enlace de restablecimiento del correo | 5- Ingresar nueva contrasena | 6- Confirmar | 7- Pulsar GUARDAR CONTRASENA</t>
+  </si>
+  <si>
+    <t>Precondiciones: Abrir la pantalla Restablecer contrasena sin un enlace valido | 1- Abrir la pantalla Restablecer contrasena sin un enlace valido | 2- Observar mensaje</t>
+  </si>
+  <si>
+    <t>Precondiciones: Usuario autenticado con cookie app_session | 1- Iniciar sesion | 2- Recargar pagina | 3- Validar que la sesion siga activa</t>
+  </si>
+  <si>
+    <t>Precondiciones: No tener cookie valida | 1- Intentar abrir Administracion | 2- Observar redireccion</t>
+  </si>
+  <si>
+    <t>Precondiciones: Usuario autenticado | 1- Abrir Mi Perfil | 2- Observar datos y resumen</t>
+  </si>
+  <si>
+    <t>Precondiciones: Usuario autenticado | 1- Abrir Mi Perfil | 2- Hacer clic en Cambiar contrasena | 3- Capturar correo de sesion | 4- Capturar password actual | 5- Capturar nuevo password | 6- Pulsar Actualizar contrasena</t>
+  </si>
+  <si>
+    <t>Precondiciones: Alumno autenticado | 1- Abrir Libros | 2- Esperar carga del catalogo | 3- Revisar listado</t>
+  </si>
+  <si>
+    <t>Precondiciones: Alumno autenticado y API no disponible | 1- Abrir Libros | 2- Simular error de backend</t>
+  </si>
+  <si>
+    <t>Precondiciones: Alumno con documentos habilitados y menos de 3 solicitudes activas | 1- Abrir Libros | 2- Seleccionar libro disponible | 3- Pulsar Solicitar | 4- Confirmar modal</t>
+  </si>
+  <si>
+    <t>Precondiciones: Alumno tiene_documentos=false | 1- Abrir Libros | 2- Intentar solicitar libro</t>
+  </si>
+  <si>
+    <t>Precondiciones: Alumno con 3 solicitudes activas | 1- Abrir Libros | 2- Intentar solicitar otro libro</t>
+  </si>
+  <si>
+    <t>Precondiciones: Alumno con solicitud cancelable | 1- Abrir Mis solicitudes de libros | 2- Seleccionar solicitud pendiente | 3- Pulsar Cancelar | 4- Confirmar</t>
+  </si>
+  <si>
+    <t>Precondiciones: Admin autenticado | 1- Abrir Libros | 2- Capturar datos de libro | 3- Capturar datos de ejemplar | 4- Pulsar Guardar</t>
+  </si>
+  <si>
+    <t>Precondiciones: Admin autenticado | 1- Abrir Alumnos | 2- Capturar boleta | 3- Capturar nombre | 4- Capturar grupo | 5- Pulsar Guardar</t>
+  </si>
+  <si>
+    <t>Precondiciones: Admin autenticado con archivo XLSX | 1- Abrir Alumnos | 2- Hacer clic en Carga masiva | 3- Seleccionar XLSX | 4- Esperar vista previa</t>
+  </si>
+  <si>
+    <t>Precondiciones: Admin autenticado y usuario existente | 1- Abrir Documentos | 2- Seleccionar alumno | 3- Habilitar documentacion</t>
+  </si>
+  <si>
+    <t>Precondiciones: Admin autenticado y alumno con documentos | 1- Abrir Solicitudes de libros | 2- Seleccionar solicitud | 3- Elegir Aprobar | 4- Confirmar</t>
+  </si>
+  <si>
+    <t>Precondiciones: Solicitud aprobada y ejemplar disponible | 1- Abrir Solicitudes de libros | 2- Seleccionar solicitud aprobada | 3- Registrar entrega | 4- Confirmar</t>
+  </si>
+  <si>
+    <t>Precondiciones: Admin autenticado | 1- Abrir Prestamos Libros | 2- Observar listado</t>
+  </si>
+  <si>
+    <t>Precondiciones: Admin autenticado | 1- Abrir Analytics | 2- Esperar carga</t>
+  </si>
+  <si>
+    <t>Precondiciones: Admin autenticado con datos cargados | 1- Abrir Reportes | 2- Hacer clic en Exportar PDF o Exportar Excel</t>
+  </si>
+  <si>
+    <t>Precondiciones: Usuario autenticado | 1- Hacer clic en Soporte | 2- Elegir Reportar error | 3- Seleccionar tipo | 4- Ingresar modulo, titulo y descripcion | 5- Pulsar Enviar</t>
+  </si>
+  <si>
+    <t>Precondiciones: Usuario sin sesion | 1- Abrir Reportar error | 2- Capturar correo y nombre | 3- Completar incidencia | 4- Enviar</t>
+  </si>
+  <si>
+    <t>Precondiciones: Usuario support_admin/support_agent autenticado | 1- Abrir Tickets | 2- Aplicar filtros | 3- Observar resultados</t>
+  </si>
+  <si>
+    <t>Precondiciones: Sesion support_admin | 1- Abrir Agregar agente de soporte | 2- Capturar nombre | 3- Capturar correo | 4- Capturar boleta opcional | 5- Capturar password y confirmacion | 6- Pulsar Guardar</t>
+  </si>
+  <si>
+    <t>Precondiciones: Sesion support_agent | 1- Intentar abrir Agregar agente de soporte | 2- Intentar guardar un agente nuevo</t>
   </si>
 </sst>
 </file>
@@ -1773,6 +1661,9 @@
     <xf numFmtId="0" fontId="6" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1780,9 +1671,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2361,40 +2249,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="35.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13"/>
-      <c r="H1" s="13"/>
-      <c r="I1" s="13"/>
-      <c r="J1" s="14"/>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
+      <c r="G1" s="14"/>
+      <c r="H1" s="14"/>
+      <c r="I1" s="14"/>
+      <c r="J1" s="15"/>
     </row>
     <row r="2" spans="1:10" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="15" t="s">
+      <c r="A2" s="16" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="14"/>
-      <c r="C2" s="15" t="s">
+      <c r="B2" s="15"/>
+      <c r="C2" s="16" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="14"/>
-      <c r="E2" s="15" t="s">
+      <c r="D2" s="15"/>
+      <c r="E2" s="16" t="s">
         <v>3</v>
       </c>
-      <c r="F2" s="14"/>
-      <c r="G2" s="15" t="s">
+      <c r="F2" s="15"/>
+      <c r="G2" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="H2" s="14"/>
-      <c r="I2" s="15" t="s">
+      <c r="H2" s="15"/>
+      <c r="I2" s="16" t="s">
         <v>5</v>
       </c>
-      <c r="J2" s="14"/>
+      <c r="J2" s="15"/>
     </row>
     <row r="3" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
@@ -2428,7 +2316,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="114.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" ht="63.75" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>16</v>
       </c>
@@ -2439,121 +2327,121 @@
         <v>18</v>
       </c>
       <c r="D4" s="4" t="s">
+        <v>396</v>
+      </c>
+      <c r="E4" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="F4" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="F4" s="4" t="s">
+      <c r="G4" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="G4" s="4" t="s">
+      <c r="H4" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="H4" s="7" t="s">
+      <c r="I4" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="I4" s="7" t="s">
+      <c r="J4" s="8" t="s">
         <v>24</v>
-      </c>
-      <c r="J4" s="8" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="51" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="B5" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="C5" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="D5" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="E5" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="E5" s="6" t="s">
+      <c r="F5" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="F5" s="6" t="s">
+      <c r="G5" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="G5" s="6" t="s">
+      <c r="H5" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="H5" s="9" t="s">
+      <c r="I5" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="I5" s="9" t="s">
+      <c r="J5" s="10" t="s">
         <v>34</v>
-      </c>
-      <c r="J5" s="10" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="63.75" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B6" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="C6" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="D6" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="E6" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="E6" s="4" t="s">
+      <c r="F6" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="F6" s="4" t="s">
+      <c r="G6" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="G6" s="4" t="s">
+      <c r="H6" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="H6" s="7" t="s">
-        <v>43</v>
-      </c>
       <c r="I6" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="J6" s="10" t="s">
         <v>34</v>
-      </c>
-      <c r="J6" s="10" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="7" spans="1:10" ht="63.75" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="B7" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="C7" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="D7" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="C7" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="D7" s="6" t="s">
+      <c r="E7" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E7" s="6" t="s">
+      <c r="F7" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="F7" s="6" t="s">
+      <c r="G7" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="G7" s="6" t="s">
+      <c r="H7" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="H7" s="9" t="s">
-        <v>50</v>
-      </c>
       <c r="I7" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="J7" s="10" t="s">
         <v>34</v>
-      </c>
-      <c r="J7" s="10" t="s">
-        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -2586,40 +2474,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="35.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13"/>
-      <c r="H1" s="13"/>
-      <c r="I1" s="13"/>
-      <c r="J1" s="14"/>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
+      <c r="G1" s="14"/>
+      <c r="H1" s="14"/>
+      <c r="I1" s="14"/>
+      <c r="J1" s="15"/>
     </row>
     <row r="2" spans="1:10" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="15" t="s">
-        <v>237</v>
-      </c>
-      <c r="B2" s="14"/>
-      <c r="C2" s="15" t="s">
-        <v>238</v>
-      </c>
-      <c r="D2" s="14"/>
-      <c r="E2" s="15" t="s">
-        <v>239</v>
-      </c>
-      <c r="F2" s="14"/>
-      <c r="G2" s="15" t="s">
+      <c r="A2" s="16" t="s">
+        <v>218</v>
+      </c>
+      <c r="B2" s="15"/>
+      <c r="C2" s="16" t="s">
+        <v>219</v>
+      </c>
+      <c r="D2" s="15"/>
+      <c r="E2" s="16" t="s">
+        <v>220</v>
+      </c>
+      <c r="F2" s="15"/>
+      <c r="G2" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="H2" s="14"/>
-      <c r="I2" s="15" t="s">
+      <c r="H2" s="15"/>
+      <c r="I2" s="16" t="s">
         <v>5</v>
       </c>
-      <c r="J2" s="14"/>
+      <c r="J2" s="15"/>
     </row>
     <row r="3" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
@@ -2655,130 +2543,130 @@
     </row>
     <row r="4" spans="1:10" ht="170.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>240</v>
+        <v>221</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>241</v>
+        <v>222</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>18</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>242</v>
+        <v>415</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>243</v>
+        <v>223</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>244</v>
+        <v>224</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>245</v>
+        <v>225</v>
       </c>
       <c r="H4" s="7" t="s">
-        <v>246</v>
+        <v>226</v>
       </c>
       <c r="I4" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="J4" s="10" t="s">
         <v>34</v>
-      </c>
-      <c r="J4" s="10" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="170.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>247</v>
+        <v>227</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>248</v>
+        <v>228</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>249</v>
+        <v>229</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>250</v>
+        <v>230</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>251</v>
+        <v>231</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>252</v>
+        <v>232</v>
       </c>
       <c r="H5" s="9" t="s">
-        <v>253</v>
+        <v>233</v>
       </c>
       <c r="I5" s="9" t="s">
-        <v>197</v>
+        <v>181</v>
       </c>
       <c r="J5" s="11" t="s">
-        <v>198</v>
+        <v>182</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="170.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>254</v>
+        <v>234</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>255</v>
+        <v>235</v>
       </c>
       <c r="C6" s="3" t="s">
         <v>18</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>256</v>
+        <v>416</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>257</v>
+        <v>236</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>258</v>
+        <v>237</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>259</v>
+        <v>238</v>
       </c>
       <c r="H6" s="7" t="s">
-        <v>260</v>
+        <v>239</v>
       </c>
       <c r="I6" s="7" t="s">
-        <v>197</v>
+        <v>181</v>
       </c>
       <c r="J6" s="11" t="s">
-        <v>198</v>
+        <v>182</v>
       </c>
     </row>
     <row r="7" spans="1:10" ht="170.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
-        <v>261</v>
+        <v>240</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>262</v>
+        <v>241</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>263</v>
+        <v>242</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>264</v>
+        <v>243</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>265</v>
+        <v>244</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>266</v>
+        <v>245</v>
       </c>
       <c r="H7" s="9" t="s">
-        <v>267</v>
+        <v>246</v>
       </c>
       <c r="I7" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="J7" s="10" t="s">
         <v>34</v>
-      </c>
-      <c r="J7" s="10" t="s">
-        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -2812,40 +2700,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="35.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13"/>
-      <c r="H1" s="13"/>
-      <c r="I1" s="13"/>
-      <c r="J1" s="14"/>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
+      <c r="G1" s="14"/>
+      <c r="H1" s="14"/>
+      <c r="I1" s="14"/>
+      <c r="J1" s="15"/>
     </row>
     <row r="2" spans="1:10" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="15" t="s">
-        <v>268</v>
-      </c>
-      <c r="B2" s="14"/>
-      <c r="C2" s="15" t="s">
-        <v>269</v>
-      </c>
-      <c r="D2" s="14"/>
-      <c r="E2" s="15" t="s">
-        <v>270</v>
-      </c>
-      <c r="F2" s="14"/>
-      <c r="G2" s="15" t="s">
+      <c r="A2" s="16" t="s">
+        <v>247</v>
+      </c>
+      <c r="B2" s="15"/>
+      <c r="C2" s="16" t="s">
+        <v>248</v>
+      </c>
+      <c r="D2" s="15"/>
+      <c r="E2" s="16" t="s">
+        <v>249</v>
+      </c>
+      <c r="F2" s="15"/>
+      <c r="G2" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="H2" s="14"/>
-      <c r="I2" s="15" t="s">
+      <c r="H2" s="15"/>
+      <c r="I2" s="16" t="s">
         <v>5</v>
       </c>
-      <c r="J2" s="14"/>
+      <c r="J2" s="15"/>
     </row>
     <row r="3" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
@@ -2881,66 +2769,66 @@
     </row>
     <row r="4" spans="1:10" ht="170.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>271</v>
+        <v>250</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>272</v>
+        <v>251</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>18</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>273</v>
+        <v>417</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>274</v>
+        <v>252</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>275</v>
+        <v>253</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>276</v>
+        <v>254</v>
       </c>
       <c r="H4" s="7" t="s">
-        <v>277</v>
+        <v>255</v>
       </c>
       <c r="I4" s="7" t="s">
-        <v>197</v>
+        <v>181</v>
       </c>
       <c r="J4" s="11" t="s">
-        <v>198</v>
+        <v>182</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="170.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>278</v>
+        <v>256</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>279</v>
+        <v>257</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>280</v>
+        <v>258</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>281</v>
+        <v>259</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>282</v>
+        <v>260</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>283</v>
+        <v>261</v>
       </c>
       <c r="H5" s="9" t="s">
-        <v>284</v>
+        <v>262</v>
       </c>
       <c r="I5" s="9" t="s">
-        <v>197</v>
+        <v>181</v>
       </c>
       <c r="J5" s="11" t="s">
-        <v>198</v>
+        <v>182</v>
       </c>
     </row>
   </sheetData>
@@ -2974,40 +2862,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="35.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13"/>
-      <c r="H1" s="13"/>
-      <c r="I1" s="13"/>
-      <c r="J1" s="14"/>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
+      <c r="G1" s="14"/>
+      <c r="H1" s="14"/>
+      <c r="I1" s="14"/>
+      <c r="J1" s="15"/>
     </row>
     <row r="2" spans="1:10" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="15" t="s">
-        <v>285</v>
-      </c>
-      <c r="B2" s="14"/>
-      <c r="C2" s="15" t="s">
-        <v>286</v>
-      </c>
-      <c r="D2" s="14"/>
-      <c r="E2" s="15" t="s">
-        <v>287</v>
-      </c>
-      <c r="F2" s="14"/>
-      <c r="G2" s="15" t="s">
+      <c r="A2" s="16" t="s">
+        <v>263</v>
+      </c>
+      <c r="B2" s="15"/>
+      <c r="C2" s="16" t="s">
+        <v>264</v>
+      </c>
+      <c r="D2" s="15"/>
+      <c r="E2" s="16" t="s">
+        <v>265</v>
+      </c>
+      <c r="F2" s="15"/>
+      <c r="G2" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="H2" s="14"/>
-      <c r="I2" s="15" t="s">
+      <c r="H2" s="15"/>
+      <c r="I2" s="16" t="s">
         <v>5</v>
       </c>
-      <c r="J2" s="14"/>
+      <c r="J2" s="15"/>
     </row>
     <row r="3" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
@@ -3043,98 +2931,98 @@
     </row>
     <row r="4" spans="1:10" ht="170.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>288</v>
+        <v>266</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>289</v>
+        <v>267</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>18</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>290</v>
+        <v>418</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>291</v>
+        <v>268</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>292</v>
+        <v>269</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>293</v>
+        <v>270</v>
       </c>
       <c r="H4" s="7" t="s">
-        <v>294</v>
+        <v>271</v>
       </c>
       <c r="I4" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="J4" s="10" t="s">
         <v>34</v>
-      </c>
-      <c r="J4" s="10" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="170.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>295</v>
+        <v>272</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>296</v>
+        <v>273</v>
       </c>
       <c r="C5" s="5" t="s">
         <v>18</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>297</v>
+        <v>274</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>298</v>
+        <v>275</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>299</v>
+        <v>276</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>300</v>
+        <v>277</v>
       </c>
       <c r="H5" s="9" t="s">
-        <v>301</v>
+        <v>278</v>
       </c>
       <c r="I5" s="9" t="s">
-        <v>197</v>
+        <v>181</v>
       </c>
       <c r="J5" s="11" t="s">
-        <v>198</v>
+        <v>182</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="170.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>302</v>
+        <v>279</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>303</v>
+        <v>280</v>
       </c>
       <c r="C6" s="3" t="s">
         <v>18</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>304</v>
+        <v>419</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>305</v>
+        <v>281</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>306</v>
+        <v>282</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>307</v>
+        <v>283</v>
       </c>
       <c r="H6" s="7" t="s">
-        <v>308</v>
+        <v>284</v>
       </c>
       <c r="I6" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="J6" s="10" t="s">
         <v>34</v>
-      </c>
-      <c r="J6" s="10" t="s">
-        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -3168,40 +3056,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="35.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13"/>
-      <c r="H1" s="13"/>
-      <c r="I1" s="13"/>
-      <c r="J1" s="14"/>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
+      <c r="G1" s="14"/>
+      <c r="H1" s="14"/>
+      <c r="I1" s="14"/>
+      <c r="J1" s="15"/>
     </row>
     <row r="2" spans="1:10" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="15" t="s">
-        <v>309</v>
-      </c>
-      <c r="B2" s="14"/>
-      <c r="C2" s="15" t="s">
-        <v>310</v>
-      </c>
-      <c r="D2" s="14"/>
-      <c r="E2" s="15" t="s">
-        <v>311</v>
-      </c>
-      <c r="F2" s="14"/>
-      <c r="G2" s="15" t="s">
+      <c r="A2" s="16" t="s">
+        <v>285</v>
+      </c>
+      <c r="B2" s="15"/>
+      <c r="C2" s="16" t="s">
+        <v>286</v>
+      </c>
+      <c r="D2" s="15"/>
+      <c r="E2" s="16" t="s">
+        <v>287</v>
+      </c>
+      <c r="F2" s="15"/>
+      <c r="G2" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="H2" s="14"/>
-      <c r="I2" s="15" t="s">
+      <c r="H2" s="15"/>
+      <c r="I2" s="16" t="s">
         <v>5</v>
       </c>
-      <c r="J2" s="14"/>
+      <c r="J2" s="15"/>
     </row>
     <row r="3" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
@@ -3237,66 +3125,66 @@
     </row>
     <row r="4" spans="1:10" ht="170.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>312</v>
+        <v>288</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>313</v>
+        <v>289</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>18</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>314</v>
+        <v>420</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>315</v>
+        <v>290</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>316</v>
+        <v>291</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>317</v>
+        <v>292</v>
       </c>
       <c r="H4" s="7" t="s">
-        <v>318</v>
+        <v>293</v>
       </c>
       <c r="I4" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="J4" s="10" t="s">
         <v>34</v>
-      </c>
-      <c r="J4" s="10" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="170.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>319</v>
+        <v>294</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>320</v>
+        <v>295</v>
       </c>
       <c r="C5" s="5" t="s">
         <v>18</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>321</v>
+        <v>296</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>322</v>
+        <v>297</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>323</v>
+        <v>298</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>324</v>
+        <v>299</v>
       </c>
       <c r="H5" s="9" t="s">
-        <v>325</v>
+        <v>300</v>
       </c>
       <c r="I5" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="J5" s="10" t="s">
         <v>34</v>
-      </c>
-      <c r="J5" s="10" t="s">
-        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -3329,40 +3217,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="35.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13"/>
-      <c r="H1" s="13"/>
-      <c r="I1" s="13"/>
-      <c r="J1" s="14"/>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
+      <c r="G1" s="14"/>
+      <c r="H1" s="14"/>
+      <c r="I1" s="14"/>
+      <c r="J1" s="15"/>
     </row>
     <row r="2" spans="1:10" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="15" t="s">
-        <v>326</v>
-      </c>
-      <c r="B2" s="14"/>
-      <c r="C2" s="15" t="s">
-        <v>327</v>
-      </c>
-      <c r="D2" s="14"/>
-      <c r="E2" s="15" t="s">
-        <v>328</v>
-      </c>
-      <c r="F2" s="14"/>
-      <c r="G2" s="15" t="s">
+      <c r="A2" s="16" t="s">
+        <v>301</v>
+      </c>
+      <c r="B2" s="15"/>
+      <c r="C2" s="16" t="s">
+        <v>302</v>
+      </c>
+      <c r="D2" s="15"/>
+      <c r="E2" s="16" t="s">
+        <v>303</v>
+      </c>
+      <c r="F2" s="15"/>
+      <c r="G2" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="H2" s="14"/>
-      <c r="I2" s="15" t="s">
+      <c r="H2" s="15"/>
+      <c r="I2" s="16" t="s">
         <v>5</v>
       </c>
-      <c r="J2" s="14"/>
+      <c r="J2" s="15"/>
     </row>
     <row r="3" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
@@ -3398,66 +3286,66 @@
     </row>
     <row r="4" spans="1:10" ht="170.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>329</v>
+        <v>304</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>330</v>
+        <v>305</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>18</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>331</v>
+        <v>421</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>332</v>
+        <v>306</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>316</v>
+        <v>291</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>333</v>
+        <v>307</v>
       </c>
       <c r="H4" s="7" t="s">
-        <v>334</v>
+        <v>308</v>
       </c>
       <c r="I4" s="7" t="s">
-        <v>197</v>
+        <v>181</v>
       </c>
       <c r="J4" s="11" t="s">
-        <v>198</v>
+        <v>182</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="170.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>335</v>
+        <v>309</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>336</v>
+        <v>310</v>
       </c>
       <c r="C5" s="5" t="s">
         <v>18</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>337</v>
+        <v>422</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>338</v>
+        <v>311</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>339</v>
+        <v>312</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>340</v>
+        <v>313</v>
       </c>
       <c r="H5" s="9" t="s">
-        <v>341</v>
+        <v>314</v>
       </c>
       <c r="I5" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="J5" s="10" t="s">
         <v>34</v>
-      </c>
-      <c r="J5" s="10" t="s">
-        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -3491,40 +3379,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="35.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13"/>
-      <c r="H1" s="13"/>
-      <c r="I1" s="13"/>
-      <c r="J1" s="14"/>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
+      <c r="G1" s="14"/>
+      <c r="H1" s="14"/>
+      <c r="I1" s="14"/>
+      <c r="J1" s="15"/>
     </row>
     <row r="2" spans="1:10" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="15" t="s">
-        <v>342</v>
-      </c>
-      <c r="B2" s="14"/>
-      <c r="C2" s="15" t="s">
-        <v>343</v>
-      </c>
-      <c r="D2" s="14"/>
-      <c r="E2" s="15" t="s">
-        <v>344</v>
-      </c>
-      <c r="F2" s="14"/>
-      <c r="G2" s="15" t="s">
+      <c r="A2" s="16" t="s">
+        <v>315</v>
+      </c>
+      <c r="B2" s="15"/>
+      <c r="C2" s="16" t="s">
+        <v>316</v>
+      </c>
+      <c r="D2" s="15"/>
+      <c r="E2" s="16" t="s">
+        <v>317</v>
+      </c>
+      <c r="F2" s="15"/>
+      <c r="G2" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="H2" s="14"/>
-      <c r="I2" s="15" t="s">
+      <c r="H2" s="15"/>
+      <c r="I2" s="16" t="s">
         <v>5</v>
       </c>
-      <c r="J2" s="14"/>
+      <c r="J2" s="15"/>
     </row>
     <row r="3" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
@@ -3558,100 +3446,100 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="76.5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" ht="51" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>345</v>
+        <v>318</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>346</v>
+        <v>319</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>18</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>347</v>
+        <v>423</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>348</v>
+        <v>320</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>349</v>
+        <v>321</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>350</v>
+        <v>322</v>
       </c>
       <c r="H4" s="7" t="s">
-        <v>351</v>
+        <v>323</v>
       </c>
       <c r="I4" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="J4" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="J4" s="10" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" ht="63.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="5" spans="1:10" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>352</v>
+        <v>324</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>353</v>
+        <v>325</v>
       </c>
       <c r="C5" s="5" t="s">
         <v>18</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>354</v>
+        <v>424</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>355</v>
+        <v>326</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>356</v>
+        <v>327</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>357</v>
+        <v>328</v>
       </c>
       <c r="H5" s="9" t="s">
-        <v>358</v>
+        <v>329</v>
       </c>
       <c r="I5" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="J5" s="10" t="s">
         <v>34</v>
-      </c>
-      <c r="J5" s="10" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="63.75" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>359</v>
+        <v>330</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>360</v>
+        <v>331</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>361</v>
+        <v>332</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>362</v>
+        <v>333</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>363</v>
+        <v>334</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>364</v>
+        <v>335</v>
       </c>
       <c r="H6" s="7" t="s">
-        <v>365</v>
+        <v>336</v>
       </c>
       <c r="I6" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="J6" s="10" t="s">
         <v>34</v>
-      </c>
-      <c r="J6" s="10" t="s">
-        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -3684,40 +3572,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="35.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13"/>
-      <c r="H1" s="13"/>
-      <c r="I1" s="13"/>
-      <c r="J1" s="14"/>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
+      <c r="G1" s="14"/>
+      <c r="H1" s="14"/>
+      <c r="I1" s="14"/>
+      <c r="J1" s="15"/>
     </row>
     <row r="2" spans="1:10" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="15" t="s">
-        <v>366</v>
-      </c>
-      <c r="B2" s="14"/>
-      <c r="C2" s="15" t="s">
-        <v>367</v>
-      </c>
-      <c r="D2" s="14"/>
-      <c r="E2" s="15" t="s">
-        <v>368</v>
-      </c>
-      <c r="F2" s="14"/>
-      <c r="G2" s="15" t="s">
+      <c r="A2" s="16" t="s">
+        <v>337</v>
+      </c>
+      <c r="B2" s="15"/>
+      <c r="C2" s="16" t="s">
+        <v>338</v>
+      </c>
+      <c r="D2" s="15"/>
+      <c r="E2" s="16" t="s">
+        <v>339</v>
+      </c>
+      <c r="F2" s="15"/>
+      <c r="G2" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="H2" s="14"/>
-      <c r="I2" s="15" t="s">
+      <c r="H2" s="15"/>
+      <c r="I2" s="16" t="s">
         <v>5</v>
       </c>
-      <c r="J2" s="14"/>
+      <c r="J2" s="15"/>
     </row>
     <row r="3" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
@@ -3751,164 +3639,164 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="63.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>369</v>
+        <v>340</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>370</v>
+        <v>341</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>18</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>371</v>
+        <v>425</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>372</v>
+        <v>342</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>373</v>
+        <v>343</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>374</v>
+        <v>344</v>
       </c>
       <c r="H4" s="7" t="s">
-        <v>375</v>
+        <v>345</v>
       </c>
       <c r="I4" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="J4" s="10" t="s">
         <v>34</v>
-      </c>
-      <c r="J4" s="10" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>376</v>
+        <v>346</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>377</v>
+        <v>347</v>
       </c>
       <c r="C5" s="5" t="s">
         <v>18</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>378</v>
+        <v>348</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>379</v>
+        <v>349</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>380</v>
+        <v>350</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>381</v>
+        <v>351</v>
       </c>
       <c r="H5" s="9" t="s">
-        <v>382</v>
+        <v>352</v>
       </c>
       <c r="I5" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="J5" s="10" t="s">
         <v>34</v>
-      </c>
-      <c r="J5" s="10" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="63.75" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>383</v>
+        <v>353</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>384</v>
+        <v>354</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>385</v>
+        <v>355</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>386</v>
+        <v>356</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>387</v>
+        <v>357</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>388</v>
+        <v>358</v>
       </c>
       <c r="H6" s="7" t="s">
-        <v>389</v>
+        <v>359</v>
       </c>
       <c r="I6" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="J6" s="10" t="s">
         <v>34</v>
-      </c>
-      <c r="J6" s="10" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="7" spans="1:10" ht="170.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
-        <v>390</v>
+        <v>360</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>391</v>
+        <v>361</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>392</v>
+        <v>362</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>393</v>
+        <v>363</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>394</v>
+        <v>364</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>395</v>
+        <v>365</v>
       </c>
       <c r="H7" s="9" t="s">
-        <v>396</v>
+        <v>366</v>
       </c>
       <c r="I7" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="J7" s="10" t="s">
         <v>34</v>
-      </c>
-      <c r="J7" s="10" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="8" spans="1:10" ht="170.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>397</v>
+        <v>367</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>398</v>
+        <v>368</v>
       </c>
       <c r="C8" s="3" t="s">
         <v>18</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>399</v>
+        <v>369</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>400</v>
+        <v>370</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>401</v>
+        <v>371</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>402</v>
+        <v>372</v>
       </c>
       <c r="H8" s="7" t="s">
-        <v>403</v>
+        <v>373</v>
       </c>
       <c r="I8" s="7" t="s">
-        <v>197</v>
+        <v>181</v>
       </c>
       <c r="J8" s="11" t="s">
-        <v>198</v>
+        <v>182</v>
       </c>
     </row>
   </sheetData>
@@ -3942,40 +3830,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="35.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13"/>
-      <c r="H1" s="13"/>
-      <c r="I1" s="13"/>
-      <c r="J1" s="14"/>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
+      <c r="G1" s="14"/>
+      <c r="H1" s="14"/>
+      <c r="I1" s="14"/>
+      <c r="J1" s="15"/>
     </row>
     <row r="2" spans="1:10" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="15" t="s">
-        <v>404</v>
-      </c>
-      <c r="B2" s="14"/>
-      <c r="C2" s="15" t="s">
-        <v>405</v>
-      </c>
-      <c r="D2" s="14"/>
-      <c r="E2" s="15" t="s">
-        <v>406</v>
-      </c>
-      <c r="F2" s="14"/>
-      <c r="G2" s="15" t="s">
+      <c r="A2" s="16" t="s">
+        <v>374</v>
+      </c>
+      <c r="B2" s="15"/>
+      <c r="C2" s="16" t="s">
+        <v>375</v>
+      </c>
+      <c r="D2" s="15"/>
+      <c r="E2" s="16" t="s">
+        <v>376</v>
+      </c>
+      <c r="F2" s="15"/>
+      <c r="G2" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="H2" s="14"/>
-      <c r="I2" s="15" t="s">
+      <c r="H2" s="15"/>
+      <c r="I2" s="16" t="s">
         <v>5</v>
       </c>
-      <c r="J2" s="14"/>
+      <c r="J2" s="15"/>
     </row>
     <row r="3" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
@@ -4009,100 +3897,100 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="89.25" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" ht="63.75" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>407</v>
+        <v>377</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>408</v>
+        <v>378</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>18</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>409</v>
+        <v>426</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>410</v>
+        <v>379</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>411</v>
+        <v>380</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>412</v>
+        <v>381</v>
       </c>
       <c r="H4" s="7" t="s">
-        <v>413</v>
+        <v>382</v>
       </c>
       <c r="I4" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="J4" s="10" t="s">
         <v>34</v>
-      </c>
-      <c r="J4" s="10" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="51" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>414</v>
+        <v>383</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>415</v>
+        <v>384</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>416</v>
+        <v>385</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>417</v>
+        <v>386</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>418</v>
+        <v>387</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>419</v>
+        <v>388</v>
       </c>
       <c r="H5" s="9" t="s">
-        <v>420</v>
+        <v>389</v>
       </c>
       <c r="I5" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="J5" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="J5" s="10" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" ht="38.25" x14ac:dyDescent="0.25">
+    </row>
+    <row r="6" spans="1:10" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>421</v>
+        <v>390</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>422</v>
+        <v>391</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>423</v>
+        <v>427</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>424</v>
+        <v>392</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>425</v>
+        <v>393</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>426</v>
+        <v>394</v>
       </c>
       <c r="H6" s="7" t="s">
-        <v>427</v>
+        <v>395</v>
       </c>
       <c r="I6" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="J6" s="10" t="s">
         <v>34</v>
-      </c>
-      <c r="J6" s="10" t="s">
-        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -4135,40 +4023,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="35.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13"/>
-      <c r="H1" s="13"/>
-      <c r="I1" s="13"/>
-      <c r="J1" s="14"/>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
+      <c r="G1" s="14"/>
+      <c r="H1" s="14"/>
+      <c r="I1" s="14"/>
+      <c r="J1" s="15"/>
     </row>
     <row r="2" spans="1:10" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="15" t="s">
+      <c r="A2" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="B2" s="15"/>
+      <c r="C2" s="16" t="s">
         <v>51</v>
       </c>
-      <c r="B2" s="14"/>
-      <c r="C2" s="15" t="s">
+      <c r="D2" s="15"/>
+      <c r="E2" s="16" t="s">
         <v>52</v>
       </c>
-      <c r="D2" s="14"/>
-      <c r="E2" s="15" t="s">
-        <v>53</v>
-      </c>
-      <c r="F2" s="14"/>
-      <c r="G2" s="15" t="s">
+      <c r="F2" s="15"/>
+      <c r="G2" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="H2" s="14"/>
-      <c r="I2" s="15" t="s">
+      <c r="H2" s="15"/>
+      <c r="I2" s="16" t="s">
         <v>5</v>
       </c>
-      <c r="J2" s="14"/>
+      <c r="J2" s="15"/>
     </row>
     <row r="3" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
@@ -4204,130 +4092,130 @@
     </row>
     <row r="4" spans="1:10" ht="170.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="B4" s="4" t="s">
         <v>54</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>55</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>18</v>
       </c>
       <c r="D4" s="4" t="s">
+        <v>397</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="F4" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="G4" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="F4" s="4" t="s">
+      <c r="H4" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="G4" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="H4" s="7" t="s">
-        <v>60</v>
-      </c>
       <c r="I4" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="J4" s="10" t="s">
         <v>34</v>
-      </c>
-      <c r="J4" s="10" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="170.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C5" s="5" t="s">
         <v>18</v>
       </c>
       <c r="D5" s="6" t="s">
+        <v>398</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="F5" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="G5" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="E5" s="6" t="s">
+      <c r="H5" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="F5" s="6" t="s">
-        <v>65</v>
-      </c>
-      <c r="G5" s="6" t="s">
-        <v>66</v>
-      </c>
-      <c r="H5" s="9" t="s">
-        <v>67</v>
-      </c>
       <c r="I5" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="J5" s="10" t="s">
         <v>34</v>
-      </c>
-      <c r="J5" s="10" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="51" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="E6" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="F6" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="C6" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="D6" s="4" t="s">
+      <c r="G6" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="E6" s="4" t="s">
+      <c r="H6" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="F6" s="4" t="s">
+      <c r="I6" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="J6" s="10" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" ht="38.25" x14ac:dyDescent="0.25">
+      <c r="A7" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="G6" s="4" t="s">
+      <c r="B7" s="6" t="s">
         <v>73</v>
-      </c>
-      <c r="H6" s="7" t="s">
-        <v>74</v>
-      </c>
-      <c r="I6" s="7" t="s">
-        <v>34</v>
-      </c>
-      <c r="J6" s="10" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" ht="63.75" x14ac:dyDescent="0.25">
-      <c r="A7" s="5" t="s">
-        <v>75</v>
-      </c>
-      <c r="B7" s="6" t="s">
-        <v>76</v>
       </c>
       <c r="C7" s="5" t="s">
         <v>18</v>
       </c>
       <c r="D7" s="6" t="s">
+        <v>399</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="F7" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="G7" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="H7" s="9" t="s">
         <v>77</v>
       </c>
-      <c r="E7" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="F7" s="6" t="s">
-        <v>79</v>
-      </c>
-      <c r="G7" s="6" t="s">
-        <v>80</v>
-      </c>
-      <c r="H7" s="9" t="s">
-        <v>81</v>
-      </c>
       <c r="I7" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="J7" s="10" t="s">
         <v>34</v>
-      </c>
-      <c r="J7" s="10" t="s">
-        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -4360,40 +4248,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="35.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13"/>
-      <c r="H1" s="13"/>
-      <c r="I1" s="13"/>
-      <c r="J1" s="14"/>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
+      <c r="G1" s="14"/>
+      <c r="H1" s="14"/>
+      <c r="I1" s="14"/>
+      <c r="J1" s="15"/>
     </row>
     <row r="2" spans="1:10" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="15" t="s">
-        <v>82</v>
-      </c>
-      <c r="B2" s="14"/>
-      <c r="C2" s="15" t="s">
-        <v>83</v>
-      </c>
-      <c r="D2" s="14"/>
-      <c r="E2" s="15" t="s">
-        <v>84</v>
-      </c>
-      <c r="F2" s="14"/>
-      <c r="G2" s="15" t="s">
+      <c r="A2" s="16" t="s">
+        <v>78</v>
+      </c>
+      <c r="B2" s="15"/>
+      <c r="C2" s="16" t="s">
+        <v>79</v>
+      </c>
+      <c r="D2" s="15"/>
+      <c r="E2" s="16" t="s">
+        <v>80</v>
+      </c>
+      <c r="F2" s="15"/>
+      <c r="G2" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="H2" s="14"/>
-      <c r="I2" s="15" t="s">
+      <c r="H2" s="15"/>
+      <c r="I2" s="16" t="s">
         <v>5</v>
       </c>
-      <c r="J2" s="14"/>
+      <c r="J2" s="15"/>
     </row>
     <row r="3" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
@@ -4427,68 +4315,68 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="76.5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" ht="51" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>18</v>
       </c>
       <c r="D4" s="4" t="s">
+        <v>400</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="H4" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="I4" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J4" s="8" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" ht="38.25" x14ac:dyDescent="0.25">
+      <c r="A5" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="B5" s="6" t="s">
         <v>88</v>
       </c>
-      <c r="F4" s="4" t="s">
+      <c r="C5" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>401</v>
+      </c>
+      <c r="E5" s="6" t="s">
         <v>89</v>
       </c>
-      <c r="G4" s="4" t="s">
+      <c r="F5" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="H4" s="7" t="s">
+      <c r="G5" s="6" t="s">
         <v>91</v>
       </c>
-      <c r="I4" s="7" t="s">
+      <c r="H5" s="9" t="s">
+        <v>92</v>
+      </c>
+      <c r="I5" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="J5" s="8" t="s">
         <v>24</v>
-      </c>
-      <c r="J4" s="8" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" ht="51" x14ac:dyDescent="0.25">
-      <c r="A5" s="5" t="s">
-        <v>92</v>
-      </c>
-      <c r="B5" s="6" t="s">
-        <v>93</v>
-      </c>
-      <c r="C5" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="D5" s="6" t="s">
-        <v>94</v>
-      </c>
-      <c r="E5" s="6" t="s">
-        <v>95</v>
-      </c>
-      <c r="F5" s="6" t="s">
-        <v>96</v>
-      </c>
-      <c r="G5" s="6" t="s">
-        <v>97</v>
-      </c>
-      <c r="H5" s="9" t="s">
-        <v>98</v>
-      </c>
-      <c r="I5" s="9" t="s">
-        <v>24</v>
-      </c>
-      <c r="J5" s="8" t="s">
-        <v>25</v>
       </c>
     </row>
   </sheetData>
@@ -4521,40 +4409,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="35.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13"/>
-      <c r="H1" s="13"/>
-      <c r="I1" s="13"/>
-      <c r="J1" s="14"/>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
+      <c r="G1" s="14"/>
+      <c r="H1" s="14"/>
+      <c r="I1" s="14"/>
+      <c r="J1" s="15"/>
     </row>
     <row r="2" spans="1:10" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="15" t="s">
-        <v>99</v>
-      </c>
-      <c r="B2" s="14"/>
-      <c r="C2" s="15" t="s">
-        <v>100</v>
-      </c>
-      <c r="D2" s="14"/>
-      <c r="E2" s="15" t="s">
-        <v>101</v>
-      </c>
-      <c r="F2" s="14"/>
-      <c r="G2" s="15" t="s">
+      <c r="A2" s="16" t="s">
+        <v>93</v>
+      </c>
+      <c r="B2" s="15"/>
+      <c r="C2" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="D2" s="15"/>
+      <c r="E2" s="16" t="s">
+        <v>95</v>
+      </c>
+      <c r="F2" s="15"/>
+      <c r="G2" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="H2" s="14"/>
-      <c r="I2" s="15" t="s">
+      <c r="H2" s="15"/>
+      <c r="I2" s="16" t="s">
         <v>5</v>
       </c>
-      <c r="J2" s="14"/>
+      <c r="J2" s="15"/>
     </row>
     <row r="3" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
@@ -4588,100 +4476,100 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="102" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" ht="63.75" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>18</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>104</v>
+        <v>402</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>105</v>
+        <v>98</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>106</v>
+        <v>99</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>107</v>
+        <v>100</v>
       </c>
       <c r="H4" s="7" t="s">
-        <v>108</v>
+        <v>101</v>
       </c>
       <c r="I4" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J4" s="8" t="s">
         <v>24</v>
-      </c>
-      <c r="J4" s="8" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>109</v>
+        <v>102</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>110</v>
+        <v>103</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>111</v>
+        <v>104</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>112</v>
+        <v>105</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>113</v>
+        <v>106</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>114</v>
+        <v>107</v>
       </c>
       <c r="H5" s="9" t="s">
-        <v>115</v>
+        <v>108</v>
       </c>
       <c r="I5" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="J5" s="10" t="s">
         <v>34</v>
-      </c>
-      <c r="J5" s="10" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="170.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>116</v>
+        <v>109</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>117</v>
+        <v>110</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>118</v>
+        <v>403</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>120</v>
+        <v>112</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>121</v>
+        <v>113</v>
       </c>
       <c r="H6" s="7" t="s">
-        <v>122</v>
+        <v>114</v>
       </c>
       <c r="I6" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="J6" s="10" t="s">
         <v>34</v>
-      </c>
-      <c r="J6" s="10" t="s">
-        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -4714,40 +4602,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="35.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13"/>
-      <c r="H1" s="13"/>
-      <c r="I1" s="13"/>
-      <c r="J1" s="14"/>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
+      <c r="G1" s="14"/>
+      <c r="H1" s="14"/>
+      <c r="I1" s="14"/>
+      <c r="J1" s="15"/>
     </row>
     <row r="2" spans="1:10" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="15" t="s">
-        <v>123</v>
-      </c>
-      <c r="B2" s="14"/>
-      <c r="C2" s="15" t="s">
-        <v>124</v>
-      </c>
-      <c r="D2" s="14"/>
-      <c r="E2" s="15" t="s">
-        <v>125</v>
-      </c>
-      <c r="F2" s="14"/>
-      <c r="G2" s="15" t="s">
+      <c r="A2" s="16" t="s">
+        <v>115</v>
+      </c>
+      <c r="B2" s="15"/>
+      <c r="C2" s="16" t="s">
+        <v>116</v>
+      </c>
+      <c r="D2" s="15"/>
+      <c r="E2" s="16" t="s">
+        <v>117</v>
+      </c>
+      <c r="F2" s="15"/>
+      <c r="G2" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="H2" s="14"/>
-      <c r="I2" s="15" t="s">
+      <c r="H2" s="15"/>
+      <c r="I2" s="16" t="s">
         <v>5</v>
       </c>
-      <c r="J2" s="14"/>
+      <c r="J2" s="15"/>
     </row>
     <row r="3" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
@@ -4781,100 +4669,100 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="51" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>126</v>
+        <v>118</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>127</v>
+        <v>119</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>18</v>
       </c>
       <c r="D4" s="4" t="s">
+        <v>404</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="H4" s="7" t="s">
+        <v>123</v>
+      </c>
+      <c r="I4" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="J4" s="10" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A5" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>405</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>126</v>
+      </c>
+      <c r="F5" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="G5" s="6" t="s">
         <v>128</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="H5" s="9" t="s">
         <v>129</v>
       </c>
-      <c r="F4" s="4" t="s">
-        <v>130</v>
-      </c>
-      <c r="G4" s="4" t="s">
-        <v>131</v>
-      </c>
-      <c r="H4" s="7" t="s">
-        <v>132</v>
-      </c>
-      <c r="I4" s="7" t="s">
+      <c r="I5" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="J5" s="10" t="s">
         <v>34</v>
-      </c>
-      <c r="J4" s="10" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" ht="38.25" x14ac:dyDescent="0.25">
-      <c r="A5" s="5" t="s">
-        <v>133</v>
-      </c>
-      <c r="B5" s="6" t="s">
-        <v>134</v>
-      </c>
-      <c r="C5" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="D5" s="6" t="s">
-        <v>135</v>
-      </c>
-      <c r="E5" s="6" t="s">
-        <v>136</v>
-      </c>
-      <c r="F5" s="6" t="s">
-        <v>137</v>
-      </c>
-      <c r="G5" s="6" t="s">
-        <v>138</v>
-      </c>
-      <c r="H5" s="9" t="s">
-        <v>139</v>
-      </c>
-      <c r="I5" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="J5" s="10" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="51" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>140</v>
+        <v>130</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>141</v>
+        <v>131</v>
       </c>
       <c r="C6" s="3" t="s">
         <v>18</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>142</v>
+        <v>132</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>143</v>
+        <v>133</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>145</v>
+        <v>135</v>
       </c>
       <c r="H6" s="7" t="s">
-        <v>146</v>
+        <v>136</v>
       </c>
       <c r="I6" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="J6" s="10" t="s">
         <v>34</v>
-      </c>
-      <c r="J6" s="10" t="s">
-        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -4907,40 +4795,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="35.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13"/>
-      <c r="H1" s="13"/>
-      <c r="I1" s="13"/>
-      <c r="J1" s="14"/>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
+      <c r="G1" s="14"/>
+      <c r="H1" s="14"/>
+      <c r="I1" s="14"/>
+      <c r="J1" s="15"/>
     </row>
     <row r="2" spans="1:10" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="15" t="s">
-        <v>147</v>
-      </c>
-      <c r="B2" s="14"/>
-      <c r="C2" s="15" t="s">
-        <v>148</v>
-      </c>
-      <c r="D2" s="14"/>
-      <c r="E2" s="15" t="s">
-        <v>149</v>
-      </c>
-      <c r="F2" s="14"/>
-      <c r="G2" s="15" t="s">
+      <c r="A2" s="16" t="s">
+        <v>137</v>
+      </c>
+      <c r="B2" s="15"/>
+      <c r="C2" s="16" t="s">
+        <v>138</v>
+      </c>
+      <c r="D2" s="15"/>
+      <c r="E2" s="16" t="s">
+        <v>139</v>
+      </c>
+      <c r="F2" s="15"/>
+      <c r="G2" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="H2" s="14"/>
-      <c r="I2" s="15" t="s">
+      <c r="H2" s="15"/>
+      <c r="I2" s="16" t="s">
         <v>5</v>
       </c>
-      <c r="J2" s="14"/>
+      <c r="J2" s="15"/>
     </row>
     <row r="3" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
@@ -4976,66 +4864,66 @@
     </row>
     <row r="4" spans="1:10" ht="170.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>150</v>
+        <v>140</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>151</v>
+        <v>141</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>18</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>152</v>
+        <v>406</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>153</v>
+        <v>142</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>154</v>
+        <v>143</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>155</v>
+        <v>144</v>
       </c>
       <c r="H4" s="7" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="I4" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="J4" s="10" t="s">
         <v>34</v>
-      </c>
-      <c r="J4" s="10" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="170.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>157</v>
+        <v>146</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>158</v>
+        <v>147</v>
       </c>
       <c r="C5" s="5" t="s">
         <v>18</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>159</v>
+        <v>407</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>160</v>
+        <v>148</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>161</v>
+        <v>149</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>162</v>
+        <v>150</v>
       </c>
       <c r="H5" s="9" t="s">
-        <v>163</v>
+        <v>151</v>
       </c>
       <c r="I5" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="J5" s="10" t="s">
         <v>34</v>
-      </c>
-      <c r="J5" s="10" t="s">
-        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -5068,40 +4956,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="35.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13"/>
-      <c r="H1" s="13"/>
-      <c r="I1" s="13"/>
-      <c r="J1" s="14"/>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
+      <c r="G1" s="14"/>
+      <c r="H1" s="14"/>
+      <c r="I1" s="14"/>
+      <c r="J1" s="15"/>
     </row>
     <row r="2" spans="1:10" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="15" t="s">
-        <v>164</v>
-      </c>
-      <c r="B2" s="14"/>
-      <c r="C2" s="15" t="s">
-        <v>165</v>
-      </c>
-      <c r="D2" s="14"/>
-      <c r="E2" s="15" t="s">
-        <v>166</v>
-      </c>
-      <c r="F2" s="14"/>
-      <c r="G2" s="15" t="s">
+      <c r="A2" s="16" t="s">
+        <v>152</v>
+      </c>
+      <c r="B2" s="15"/>
+      <c r="C2" s="16" t="s">
+        <v>153</v>
+      </c>
+      <c r="D2" s="15"/>
+      <c r="E2" s="16" t="s">
+        <v>154</v>
+      </c>
+      <c r="F2" s="15"/>
+      <c r="G2" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="H2" s="14"/>
-      <c r="I2" s="15" t="s">
+      <c r="H2" s="15"/>
+      <c r="I2" s="16" t="s">
         <v>5</v>
       </c>
-      <c r="J2" s="14"/>
+      <c r="J2" s="15"/>
     </row>
     <row r="3" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
@@ -5137,66 +5025,66 @@
     </row>
     <row r="4" spans="1:10" ht="170.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>167</v>
+        <v>155</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>168</v>
+        <v>156</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>18</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>169</v>
+        <v>408</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>170</v>
+        <v>157</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>171</v>
+        <v>158</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>172</v>
+        <v>159</v>
       </c>
       <c r="H4" s="7" t="s">
-        <v>173</v>
+        <v>160</v>
       </c>
       <c r="I4" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="J4" s="10" t="s">
         <v>34</v>
-      </c>
-      <c r="J4" s="10" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="170.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>174</v>
+        <v>161</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>175</v>
+        <v>162</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>176</v>
+        <v>409</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>177</v>
+        <v>163</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>178</v>
+        <v>164</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>179</v>
+        <v>165</v>
       </c>
       <c r="H5" s="9" t="s">
-        <v>180</v>
+        <v>166</v>
       </c>
       <c r="I5" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="J5" s="10" t="s">
         <v>34</v>
-      </c>
-      <c r="J5" s="10" t="s">
-        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -5229,40 +5117,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="35.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13"/>
-      <c r="H1" s="13"/>
-      <c r="I1" s="13"/>
-      <c r="J1" s="14"/>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
+      <c r="G1" s="14"/>
+      <c r="H1" s="14"/>
+      <c r="I1" s="14"/>
+      <c r="J1" s="15"/>
     </row>
     <row r="2" spans="1:10" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="15" t="s">
-        <v>181</v>
-      </c>
-      <c r="B2" s="14"/>
-      <c r="C2" s="15" t="s">
-        <v>182</v>
-      </c>
-      <c r="D2" s="14"/>
-      <c r="E2" s="15" t="s">
-        <v>183</v>
-      </c>
-      <c r="F2" s="14"/>
-      <c r="G2" s="15" t="s">
+      <c r="A2" s="16" t="s">
+        <v>167</v>
+      </c>
+      <c r="B2" s="15"/>
+      <c r="C2" s="16" t="s">
+        <v>168</v>
+      </c>
+      <c r="D2" s="15"/>
+      <c r="E2" s="16" t="s">
+        <v>169</v>
+      </c>
+      <c r="F2" s="15"/>
+      <c r="G2" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="H2" s="14"/>
-      <c r="I2" s="15" t="s">
+      <c r="H2" s="15"/>
+      <c r="I2" s="16" t="s">
         <v>5</v>
       </c>
-      <c r="J2" s="14"/>
+      <c r="J2" s="15"/>
     </row>
     <row r="3" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
@@ -5298,128 +5186,128 @@
     </row>
     <row r="4" spans="1:10" ht="170.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>184</v>
+        <v>170</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>185</v>
+        <v>171</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>18</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>186</v>
+        <v>410</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>187</v>
+        <v>172</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>188</v>
+        <v>173</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>189</v>
+        <v>174</v>
       </c>
       <c r="H4" s="7" t="s">
-        <v>190</v>
+        <v>175</v>
       </c>
       <c r="I4" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="J4" s="10" t="s">
         <v>34</v>
-      </c>
-      <c r="J4" s="10" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="170.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>191</v>
+        <v>176</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>192</v>
+        <v>177</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>193</v>
+        <v>411</v>
       </c>
       <c r="E5" s="6"/>
       <c r="F5" s="6" t="s">
-        <v>194</v>
+        <v>178</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>195</v>
+        <v>179</v>
       </c>
       <c r="H5" s="9" t="s">
-        <v>196</v>
+        <v>180</v>
       </c>
       <c r="I5" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="J5" s="12" t="s">
         <v>34</v>
-      </c>
-      <c r="J5" s="16" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="170.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>199</v>
+        <v>183</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>200</v>
+        <v>184</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>201</v>
+        <v>412</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>202</v>
+        <v>185</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>203</v>
+        <v>186</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>204</v>
+        <v>187</v>
       </c>
       <c r="H6" s="7" t="s">
-        <v>205</v>
+        <v>188</v>
       </c>
       <c r="I6" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="J6" s="10" t="s">
         <v>34</v>
-      </c>
-      <c r="J6" s="10" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="7" spans="1:10" ht="170.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
-        <v>206</v>
+        <v>189</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>207</v>
+        <v>190</v>
       </c>
       <c r="C7" s="5" t="s">
         <v>18</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>208</v>
+        <v>413</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>209</v>
+        <v>191</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>210</v>
+        <v>192</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>211</v>
+        <v>193</v>
       </c>
       <c r="H7" s="9" t="s">
-        <v>212</v>
+        <v>194</v>
       </c>
       <c r="I7" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="J7" s="10" t="s">
         <v>34</v>
-      </c>
-      <c r="J7" s="10" t="s">
-        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -5452,40 +5340,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="35.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13"/>
-      <c r="H1" s="13"/>
-      <c r="I1" s="13"/>
-      <c r="J1" s="14"/>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
+      <c r="G1" s="14"/>
+      <c r="H1" s="14"/>
+      <c r="I1" s="14"/>
+      <c r="J1" s="15"/>
     </row>
     <row r="2" spans="1:10" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="15" t="s">
-        <v>213</v>
-      </c>
-      <c r="B2" s="14"/>
-      <c r="C2" s="15" t="s">
-        <v>214</v>
-      </c>
-      <c r="D2" s="14"/>
-      <c r="E2" s="15" t="s">
-        <v>215</v>
-      </c>
-      <c r="F2" s="14"/>
-      <c r="G2" s="15" t="s">
+      <c r="A2" s="16" t="s">
+        <v>195</v>
+      </c>
+      <c r="B2" s="15"/>
+      <c r="C2" s="16" t="s">
+        <v>196</v>
+      </c>
+      <c r="D2" s="15"/>
+      <c r="E2" s="16" t="s">
+        <v>197</v>
+      </c>
+      <c r="F2" s="15"/>
+      <c r="G2" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="H2" s="14"/>
-      <c r="I2" s="15" t="s">
+      <c r="H2" s="15"/>
+      <c r="I2" s="16" t="s">
         <v>5</v>
       </c>
-      <c r="J2" s="14"/>
+      <c r="J2" s="15"/>
     </row>
     <row r="3" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
@@ -5521,98 +5409,98 @@
     </row>
     <row r="4" spans="1:10" ht="170.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>216</v>
+        <v>198</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>217</v>
+        <v>199</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>18</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>218</v>
+        <v>414</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>219</v>
+        <v>200</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>220</v>
+        <v>201</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>221</v>
+        <v>202</v>
       </c>
       <c r="H4" s="7" t="s">
-        <v>222</v>
+        <v>203</v>
       </c>
       <c r="I4" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="J4" s="10" t="s">
         <v>34</v>
-      </c>
-      <c r="J4" s="10" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="170.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>223</v>
+        <v>204</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>224</v>
+        <v>205</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>225</v>
+        <v>206</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>226</v>
+        <v>207</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>227</v>
+        <v>208</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>228</v>
+        <v>209</v>
       </c>
       <c r="H5" s="9" t="s">
-        <v>229</v>
+        <v>210</v>
       </c>
       <c r="I5" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="J5" s="10" t="s">
         <v>34</v>
-      </c>
-      <c r="J5" s="10" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="170.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>230</v>
+        <v>211</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>231</v>
+        <v>212</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>232</v>
+        <v>213</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>233</v>
+        <v>214</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>234</v>
+        <v>215</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>235</v>
+        <v>216</v>
       </c>
       <c r="H6" s="7" t="s">
-        <v>236</v>
+        <v>217</v>
       </c>
       <c r="I6" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="J6" s="10" t="s">
         <v>34</v>
-      </c>
-      <c r="J6" s="10" t="s">
-        <v>35</v>
       </c>
     </row>
   </sheetData>

</xml_diff>